<commit_message>
Format picker: "and" labels, one typical-length style, lowercase list
Family labels and the reach chip say "and" instead of "&" (the
sitewide rule), with GROUP_COLORS rekeyed to match. Typical lengths
use "to" for ranges and drop closing periods. The modal's objectives
list lowercases every item after the first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/formatpicker/data/delivery_formats.xlsx
+++ b/formatpicker/data/delivery_formats.xlsx
@@ -927,7 +927,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>20+ pages</t>
+          <t>20 or more pages</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Brief &amp; summary</t>
+          <t>Brief and summary</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2-4 pages</t>
+          <t>2 to 4 pages</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>15-40 pages</t>
+          <t>15 to 40 pages</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Brief &amp; summary</t>
+          <t>Brief and summary</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1-2 pages</t>
+          <t>1 to 2 pages</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Brief &amp; summary</t>
+          <t>Brief and summary</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>10-25 slides</t>
+          <t>10 to 25 slides</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>10-45 minutes</t>
+          <t>10 to 45 minutes</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Digital &amp; interactive</t>
+          <t>Digital and interactive</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Ongoing / interactive</t>
+          <t>Ongoing and interactive</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Digital &amp; interactive</t>
+          <t>Digital and interactive</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1-2 pages or a pitch</t>
+          <t>1 to 2 pages or a pitch</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1-3 short sections</t>
+          <t>1 to 3 short sections</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>5-20 pages</t>
+          <t>5 to 20 pages</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Digital &amp; interactive</t>
+          <t>Digital and interactive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2-20 minutes</t>
+          <t>2 to 20 minutes</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>5-15 pages</t>
+          <t>5 to 15 pages</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Half a day to a full day, in person or small-group virtual.</t>
+          <t>Half a day to a full day, in person or small-group virtual</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>45 to 60 minutes, live, often recorded.</t>
+          <t>45 to 60 minutes, live, often recorded</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>One board, roughly 36 by 48 inches.</t>
+          <t>One board, roughly 36 by 48 inches</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Outreach &amp; media</t>
+          <t>Outreach and media</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>600 to 800 words.</t>
+          <t>600 to 800 words</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">

</xml_diff>

<commit_message>
Format picker: reach reason says what the format is for
The "Adapt for reach" reason strung reach labels together ("built for
both internal and external or external reach"). It now reads "Annual
Report is built to reach outside your court, so using it inside your
court means adapting how it is polished and shared", with the two
"built" and three "using" phrases as Copy rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/formatpicker/data/delivery_formats.xlsx
+++ b/formatpicker/data/delivery_formats.xlsx
@@ -2283,7 +2283,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>{format} is built for {needed} reach, so reaching {have} means adapting how it is polished and shared.</t>
+          <t>{format} is built {needed}, so {have} means adapting how it is polished and shared.</t>
         </is>
       </c>
     </row>
@@ -2787,6 +2787,66 @@
       <c r="B42" t="inlineStr">
         <is>
           <t>Different objective</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>reach_built_inside</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>for use inside your court</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>reach_built_outside</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>to reach outside your court</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>reach_use_internal</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>using it inside your court</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>reach_use_external</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>taking it outside your court</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>reach_use_both</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>using it both inside and outside your court</t>
         </is>
       </c>
     </row>

</xml_diff>